<commit_message>
Updated programme and fixed errors in parser.py
</commit_message>
<xml_diff>
--- a/programme-parser/programme.xlsx
+++ b/programme-parser/programme.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="35">
   <si>
     <t xml:space="preserve">Starttime</t>
   </si>
@@ -73,6 +73,15 @@
     <t xml:space="preserve">Eten @ Bolk</t>
   </si>
   <si>
+    <t xml:space="preserve">Bierviltjesoorlog</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dozenfort</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Speurtocht (VVT)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Weerwolven</t>
   </si>
   <si>
@@ -82,31 +91,22 @@
     <t xml:space="preserve">Sterrenkijken (VVT)</t>
   </si>
   <si>
-    <t xml:space="preserve">Bierviltjesoorlog</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dozenfort</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Speurtocht (VVT)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Band op de boot</t>
   </si>
   <si>
+    <t xml:space="preserve">Kijken hoe het klinkt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deken is lava (VVT)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Retrogames</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spelletjesavond</t>
+  </si>
+  <si>
     <t xml:space="preserve">Karaoke cocktailnight</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Retrogames</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Spelletjesavond</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Deken is lava (VVT)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kijken hoe het klinkt</t>
   </si>
   <si>
     <t xml:space="preserve">SpeBi proeverij</t>
@@ -135,7 +135,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="hh:mm:ss"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -164,12 +164,6 @@
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="0"/>
     </font>
   </fonts>
   <fills count="2">
@@ -214,40 +208,48 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -444,10 +446,10 @@
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="1" width="11.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="3" style="0" width="11.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="14" style="0" width="8.63"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="15.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="30" min="17" style="0" width="8.63"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="3" style="2" width="11.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="14" style="2" width="8.63"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="2" width="15.11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="30" min="17" style="2" width="8.63"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -457,30 +459,30 @@
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2" t="s">
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-      <c r="I1" s="2" t="s">
+      <c r="G1" s="3"/>
+      <c r="H1" s="3"/>
+      <c r="I1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="J1" s="2"/>
-      <c r="K1" s="2"/>
-      <c r="L1" s="2" t="s">
+      <c r="J1" s="3"/>
+      <c r="K1" s="3"/>
+      <c r="L1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="M1" s="2"/>
-      <c r="N1" s="2"/>
-      <c r="P1" s="0" t="s">
+      <c r="M1" s="3"/>
+      <c r="N1" s="3"/>
+      <c r="P1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="Q1" s="0" t="n">
+      <c r="Q1" s="2" t="n">
         <v>30</v>
       </c>
     </row>
@@ -489,38 +491,38 @@
         <f aca="false">TIME(17,0,0)</f>
         <v>0.708333333333333</v>
       </c>
-      <c r="B2" s="3" t="n">
+      <c r="B2" s="4" t="n">
         <f aca="false">A2+TIME(0,$Q$1,0)</f>
         <v>0.729166666666667</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4" t="s">
+      <c r="G2" s="5"/>
+      <c r="H2" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="I2" s="4" t="s">
+      <c r="I2" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="J2" s="4"/>
-      <c r="K2" s="4" t="s">
+      <c r="J2" s="5"/>
+      <c r="K2" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="L2" s="4" t="s">
+      <c r="L2" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="M2" s="4"/>
-      <c r="N2" s="4" t="s">
+      <c r="M2" s="5"/>
+      <c r="N2" s="5" t="s">
         <v>15</v>
       </c>
     </row>
@@ -529,44 +531,45 @@
         <f aca="false">A2+TIME(0,$Q$1,0)</f>
         <v>0.729166666666667</v>
       </c>
-      <c r="B3" s="3" t="n">
+      <c r="B3" s="4" t="n">
         <f aca="false">A3+TIME(0,$Q$1,0)</f>
         <v>0.75</v>
       </c>
-      <c r="C3" s="4"/>
-      <c r="D3" s="4"/>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
-      <c r="G3" s="4"/>
-      <c r="H3" s="4"/>
-      <c r="I3" s="4"/>
-      <c r="J3" s="4"/>
-      <c r="K3" s="4"/>
-      <c r="L3" s="4"/>
-      <c r="M3" s="4"/>
-      <c r="N3" s="4"/>
+      <c r="C3" s="5"/>
+      <c r="D3" s="5"/>
+      <c r="E3" s="5"/>
+      <c r="F3" s="5"/>
+      <c r="G3" s="5"/>
+      <c r="H3" s="5"/>
+      <c r="I3" s="5"/>
+      <c r="J3" s="5"/>
+      <c r="K3" s="5"/>
+      <c r="L3" s="5"/>
+      <c r="M3" s="5"/>
+      <c r="N3" s="5"/>
     </row>
     <row r="4" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="n">
         <f aca="false">A3+TIME(0,30,0)</f>
         <v>0.75</v>
       </c>
-      <c r="B4" s="3" t="n">
+      <c r="B4" s="4" t="n">
         <f aca="false">A4+TIME(0,$Q$1,0)</f>
         <v>0.770833333333333</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="D4" s="4"/>
-      <c r="E4" s="4"/>
+      <c r="D4" s="5"/>
+      <c r="E4" s="5"/>
       <c r="F4" s="5" t="s">
         <v>16</v>
       </c>
       <c r="G4" s="5"/>
-      <c r="I4" s="4"/>
-      <c r="J4" s="4"/>
-      <c r="K4" s="4"/>
+      <c r="H4" s="5"/>
+      <c r="I4" s="5"/>
+      <c r="J4" s="5"/>
+      <c r="K4" s="5"/>
       <c r="L4" s="5" t="s">
         <v>16</v>
       </c>
@@ -578,19 +581,22 @@
         <f aca="false">A4+TIME(0,30,0)</f>
         <v>0.770833333333333</v>
       </c>
-      <c r="B5" s="3" t="n">
+      <c r="B5" s="4" t="n">
         <f aca="false">A5+TIME(0,$Q$1,0)</f>
         <v>0.791666666666667</v>
       </c>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="4"/>
+      <c r="C5" s="5"/>
+      <c r="D5" s="5"/>
+      <c r="E5" s="5"/>
       <c r="F5" s="5"/>
       <c r="G5" s="5"/>
-      <c r="I5" s="4"/>
-      <c r="J5" s="4"/>
-      <c r="K5" s="4"/>
-      <c r="L5" s="4"/>
+      <c r="H5" s="5"/>
+      <c r="I5" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="J5" s="5"/>
+      <c r="K5" s="5"/>
+      <c r="L5" s="5"/>
       <c r="M5" s="5"/>
       <c r="N5" s="5"/>
     </row>
@@ -599,19 +605,20 @@
         <f aca="false">A5+TIME(0,30,0)</f>
         <v>0.791666666666667</v>
       </c>
-      <c r="B6" s="3" t="n">
+      <c r="B6" s="4" t="n">
         <f aca="false">A6+TIME(0,$Q$1,0)</f>
         <v>0.8125</v>
       </c>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
-      <c r="E6" s="4"/>
+      <c r="C6" s="5"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="5"/>
       <c r="F6" s="5"/>
       <c r="G6" s="5"/>
-      <c r="I6" s="4"/>
-      <c r="J6" s="4"/>
-      <c r="K6" s="4"/>
-      <c r="L6" s="4"/>
+      <c r="H6" s="5"/>
+      <c r="I6" s="5"/>
+      <c r="J6" s="5"/>
+      <c r="K6" s="5"/>
+      <c r="L6" s="5"/>
       <c r="M6" s="5"/>
       <c r="N6" s="5"/>
     </row>
@@ -620,26 +627,20 @@
         <f aca="false">A6+TIME(0,30,0)</f>
         <v>0.8125</v>
       </c>
-      <c r="B7" s="3" t="n">
+      <c r="B7" s="4" t="n">
         <f aca="false">A7+TIME(0,$Q$1,0)</f>
         <v>0.833333333333333</v>
       </c>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
-      <c r="E7" s="4"/>
-      <c r="F7" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="G7" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="H7" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="I7" s="4"/>
-      <c r="J7" s="4"/>
-      <c r="K7" s="4"/>
-      <c r="L7" s="4"/>
+      <c r="C7" s="5"/>
+      <c r="D7" s="5"/>
+      <c r="E7" s="5"/>
+      <c r="F7" s="5"/>
+      <c r="G7" s="5"/>
+      <c r="H7" s="5"/>
+      <c r="I7" s="5"/>
+      <c r="J7" s="5"/>
+      <c r="K7" s="5"/>
+      <c r="L7" s="5"/>
       <c r="M7" s="5"/>
       <c r="N7" s="5"/>
     </row>
@@ -648,367 +649,388 @@
         <f aca="false">A7+TIME(0,30,0)</f>
         <v>0.833333333333333</v>
       </c>
-      <c r="B8" s="3" t="n">
+      <c r="B8" s="4" t="n">
         <f aca="false">A8+TIME(0,$Q$1,0)</f>
         <v>0.854166666666667</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F8" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="G8" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="H8" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="F8" s="4"/>
-      <c r="G8" s="4"/>
-      <c r="H8" s="4"/>
-      <c r="I8" s="5" t="s">
-        <v>16</v>
-      </c>
+      <c r="I8" s="5"/>
       <c r="J8" s="5"/>
-      <c r="L8" s="4" t="s">
+      <c r="K8" s="5"/>
+      <c r="L8" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="M8" s="4"/>
-      <c r="N8" s="4"/>
+      <c r="M8" s="5"/>
+      <c r="N8" s="5"/>
     </row>
     <row r="9" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="n">
         <f aca="false">A8+TIME(0,30,0)</f>
         <v>0.854166666666667</v>
       </c>
-      <c r="B9" s="3" t="n">
+      <c r="B9" s="4" t="n">
         <f aca="false">A9+TIME(0,$Q$1,0)</f>
         <v>0.875</v>
       </c>
-      <c r="C9" s="4"/>
-      <c r="D9" s="4"/>
-      <c r="E9" s="4"/>
-      <c r="F9" s="4" t="s">
+      <c r="C9" s="5"/>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5"/>
+      <c r="F9" s="5"/>
+      <c r="G9" s="5"/>
+      <c r="H9" s="5"/>
+      <c r="I9" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="G9" s="4"/>
-      <c r="H9" s="4"/>
-      <c r="I9" s="4"/>
       <c r="J9" s="5"/>
-      <c r="L9" s="4"/>
-      <c r="M9" s="4"/>
-      <c r="N9" s="4"/>
+      <c r="K9" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="L9" s="5"/>
+      <c r="M9" s="5"/>
+      <c r="N9" s="5"/>
     </row>
     <row r="10" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="n">
         <f aca="false">A9+TIME(0,30,0)</f>
         <v>0.875</v>
       </c>
-      <c r="B10" s="3" t="n">
+      <c r="B10" s="4" t="n">
         <f aca="false">A10+TIME(0,$Q$1,0)</f>
         <v>0.895833333333333</v>
       </c>
-      <c r="C10" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="D10" s="4" t="s">
+      <c r="C10" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="E10" s="4"/>
-      <c r="F10" s="4"/>
-      <c r="G10" s="4"/>
-      <c r="H10" s="4"/>
-      <c r="I10" s="4"/>
+      <c r="D10" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="E10" s="5"/>
+      <c r="F10" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G10" s="5"/>
+      <c r="H10" s="5"/>
+      <c r="I10" s="5"/>
       <c r="J10" s="5"/>
-      <c r="L10" s="4"/>
-      <c r="M10" s="4"/>
-      <c r="N10" s="4"/>
+      <c r="K10" s="6"/>
+      <c r="L10" s="5"/>
+      <c r="M10" s="5"/>
+      <c r="N10" s="5"/>
     </row>
     <row r="11" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="n">
         <f aca="false">A10+TIME(0,30,0)</f>
         <v>0.895833333333333</v>
       </c>
-      <c r="B11" s="3" t="n">
+      <c r="B11" s="4" t="n">
         <f aca="false">A11+TIME(0,$Q$1,0)</f>
         <v>0.916666666666667</v>
       </c>
-      <c r="C11" s="4"/>
-      <c r="D11" s="4"/>
-      <c r="E11" s="4"/>
-      <c r="F11" s="4"/>
-      <c r="G11" s="4"/>
-      <c r="H11" s="4"/>
-      <c r="I11" s="4"/>
+      <c r="C11" s="5"/>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
+      <c r="F11" s="5"/>
+      <c r="G11" s="5"/>
+      <c r="H11" s="5"/>
+      <c r="I11" s="5"/>
       <c r="J11" s="5"/>
-      <c r="K11" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="L11" s="4"/>
-      <c r="M11" s="4"/>
-      <c r="N11" s="4"/>
+      <c r="K11" s="6"/>
+      <c r="L11" s="5"/>
+      <c r="M11" s="5"/>
+      <c r="N11" s="5"/>
     </row>
     <row r="12" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="n">
         <f aca="false">A11+TIME(0,30,0)</f>
         <v>0.916666666666667</v>
       </c>
-      <c r="B12" s="3" t="n">
+      <c r="B12" s="4" t="n">
         <f aca="false">A12+TIME(0,$Q$1,0)</f>
         <v>0.9375</v>
       </c>
-      <c r="C12" s="4"/>
-      <c r="D12" s="4"/>
-      <c r="F12" s="4"/>
-      <c r="G12" s="4"/>
-      <c r="I12" s="4" t="s">
+      <c r="C12" s="5"/>
+      <c r="D12" s="5"/>
+      <c r="F12" s="5"/>
+      <c r="G12" s="5"/>
+      <c r="H12" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="J12" s="4"/>
-      <c r="K12" s="4"/>
-      <c r="L12" s="4"/>
-      <c r="M12" s="4"/>
-      <c r="N12" s="4"/>
+      <c r="I12" s="5"/>
+      <c r="J12" s="5"/>
+      <c r="K12" s="6"/>
+      <c r="L12" s="5"/>
+      <c r="M12" s="5"/>
+      <c r="N12" s="5"/>
     </row>
     <row r="13" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="n">
         <f aca="false">A12+TIME(0,30,0)</f>
         <v>0.9375</v>
       </c>
-      <c r="B13" s="3" t="n">
+      <c r="B13" s="4" t="n">
         <f aca="false">A13+TIME(0,$Q$1,0)</f>
         <v>0.958333333333333</v>
       </c>
-      <c r="C13" s="4"/>
-      <c r="D13" s="4"/>
-      <c r="F13" s="4"/>
-      <c r="G13" s="4"/>
-      <c r="I13" s="4"/>
-      <c r="J13" s="4"/>
-      <c r="K13" s="4"/>
-      <c r="L13" s="4"/>
-      <c r="M13" s="4"/>
-      <c r="N13" s="4"/>
+      <c r="C13" s="5"/>
+      <c r="D13" s="5"/>
+      <c r="F13" s="5"/>
+      <c r="G13" s="5"/>
+      <c r="H13" s="7"/>
+      <c r="I13" s="5"/>
+      <c r="J13" s="5"/>
+      <c r="K13" s="6"/>
+      <c r="L13" s="5"/>
+      <c r="M13" s="5"/>
+      <c r="N13" s="5"/>
     </row>
     <row r="14" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="n">
         <f aca="false">A13+TIME(0,30,0)</f>
         <v>0.958333333333333</v>
       </c>
-      <c r="B14" s="3" t="n">
+      <c r="B14" s="4" t="n">
         <f aca="false">A14+TIME(0,$Q$1,0)</f>
         <v>0.979166666666667</v>
       </c>
-      <c r="C14" s="4"/>
-      <c r="D14" s="4"/>
-      <c r="F14" s="4"/>
-      <c r="G14" s="4"/>
-      <c r="I14" s="4" t="s">
+      <c r="C14" s="5"/>
+      <c r="D14" s="5"/>
+      <c r="F14" s="5"/>
+      <c r="G14" s="5"/>
+      <c r="H14" s="7"/>
+      <c r="I14" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="J14" s="4"/>
-      <c r="K14" s="4" t="s">
+      <c r="J14" s="5"/>
+      <c r="K14" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="L14" s="4"/>
-      <c r="M14" s="4"/>
-      <c r="N14" s="4"/>
+      <c r="L14" s="5"/>
+      <c r="M14" s="5"/>
+      <c r="N14" s="5"/>
     </row>
     <row r="15" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="n">
         <f aca="false">A14+TIME(0,30,0)</f>
         <v>0.979166666666667</v>
       </c>
-      <c r="B15" s="3" t="n">
+      <c r="B15" s="4" t="n">
         <f aca="false">A15+TIME(0,$Q$1,0)</f>
         <v>1</v>
       </c>
-      <c r="C15" s="4"/>
-      <c r="D15" s="4"/>
-      <c r="F15" s="4"/>
-      <c r="G15" s="4"/>
-      <c r="I15" s="4"/>
-      <c r="J15" s="4"/>
-      <c r="K15" s="4"/>
-      <c r="L15" s="4"/>
-      <c r="M15" s="4"/>
-      <c r="N15" s="4"/>
+      <c r="C15" s="5"/>
+      <c r="D15" s="5"/>
+      <c r="F15" s="5"/>
+      <c r="G15" s="5"/>
+      <c r="H15" s="7"/>
+      <c r="I15" s="5"/>
+      <c r="J15" s="5"/>
+      <c r="K15" s="5"/>
+      <c r="L15" s="5"/>
+      <c r="M15" s="5"/>
+      <c r="N15" s="5"/>
     </row>
     <row r="16" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="n">
         <f aca="false">A15+TIME(0,30,0)</f>
         <v>1</v>
       </c>
-      <c r="B16" s="3" t="n">
+      <c r="B16" s="4" t="n">
         <f aca="false">A16+TIME(0,$Q$1,0)</f>
         <v>1.02083333333333</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="C16" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="D16" s="4"/>
-      <c r="E16" s="4"/>
-      <c r="F16" s="4"/>
-      <c r="G16" s="4"/>
-      <c r="I16" s="4"/>
-      <c r="J16" s="4"/>
-      <c r="K16" s="4"/>
+      <c r="D16" s="5"/>
+      <c r="E16" s="5"/>
+      <c r="F16" s="5"/>
+      <c r="G16" s="5"/>
+      <c r="H16" s="7"/>
+      <c r="I16" s="5"/>
+      <c r="J16" s="5"/>
+      <c r="K16" s="5"/>
     </row>
     <row r="17" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="n">
         <f aca="false">A16+TIME(0,30,0)</f>
         <v>1.02083333333333</v>
       </c>
-      <c r="B17" s="3" t="n">
+      <c r="B17" s="4" t="n">
         <f aca="false">A17+TIME(0,$Q$1,0)</f>
         <v>1.04166666666667</v>
       </c>
-      <c r="C17" s="4"/>
-      <c r="D17" s="4"/>
-      <c r="E17" s="4"/>
-      <c r="F17" s="4"/>
-      <c r="G17" s="4"/>
-      <c r="I17" s="4"/>
-      <c r="J17" s="4"/>
-      <c r="K17" s="4"/>
+      <c r="C17" s="5"/>
+      <c r="D17" s="5"/>
+      <c r="E17" s="5"/>
+      <c r="F17" s="5"/>
+      <c r="G17" s="5"/>
+      <c r="H17" s="7"/>
+      <c r="I17" s="5"/>
+      <c r="J17" s="5"/>
+      <c r="K17" s="5"/>
     </row>
     <row r="18" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="n">
         <f aca="false">A17+TIME(0,30,0)</f>
         <v>1.04166666666667</v>
       </c>
-      <c r="B18" s="3" t="n">
+      <c r="B18" s="4" t="n">
         <f aca="false">A18+TIME(0,$Q$1,0)</f>
         <v>1.0625</v>
       </c>
-      <c r="C18" s="4"/>
-      <c r="D18" s="4"/>
-      <c r="E18" s="4"/>
-      <c r="F18" s="4"/>
-      <c r="G18" s="4"/>
-      <c r="I18" s="4" t="s">
+      <c r="C18" s="5"/>
+      <c r="D18" s="5"/>
+      <c r="E18" s="5"/>
+      <c r="F18" s="5"/>
+      <c r="G18" s="5"/>
+      <c r="H18" s="7"/>
+      <c r="I18" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="J18" s="4"/>
-      <c r="K18" s="4"/>
+      <c r="J18" s="5"/>
+      <c r="K18" s="5"/>
     </row>
     <row r="19" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="n">
         <f aca="false">A18+TIME(0,30,0)</f>
         <v>1.0625</v>
       </c>
-      <c r="B19" s="3" t="n">
+      <c r="B19" s="4" t="n">
         <f aca="false">A19+TIME(0,$Q$1,0)</f>
         <v>1.08333333333333</v>
       </c>
-      <c r="C19" s="4"/>
-      <c r="D19" s="4"/>
-      <c r="E19" s="4"/>
-      <c r="F19" s="4"/>
-      <c r="G19" s="4"/>
-      <c r="I19" s="4" t="s">
+      <c r="C19" s="5"/>
+      <c r="D19" s="5"/>
+      <c r="E19" s="5"/>
+      <c r="F19" s="5"/>
+      <c r="G19" s="5"/>
+      <c r="H19" s="7"/>
+      <c r="I19" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="J19" s="4"/>
-      <c r="K19" s="4"/>
+      <c r="J19" s="5"/>
+      <c r="K19" s="5"/>
     </row>
     <row r="20" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="n">
         <f aca="false">A19+TIME(0,30,0)</f>
         <v>1.08333333333333</v>
       </c>
-      <c r="B20" s="3" t="n">
+      <c r="B20" s="4" t="n">
         <f aca="false">A20+TIME(0,$Q$1,0)</f>
         <v>1.10416666666667</v>
       </c>
-      <c r="C20" s="4"/>
-      <c r="D20" s="4"/>
-      <c r="E20" s="4"/>
-      <c r="F20" s="4"/>
-      <c r="G20" s="4"/>
-      <c r="I20" s="4"/>
-      <c r="J20" s="4"/>
-      <c r="K20" s="4"/>
+      <c r="C20" s="5"/>
+      <c r="D20" s="5"/>
+      <c r="E20" s="5"/>
+      <c r="F20" s="5"/>
+      <c r="G20" s="5"/>
+      <c r="H20" s="7"/>
+      <c r="I20" s="5"/>
+      <c r="J20" s="5"/>
+      <c r="K20" s="5"/>
     </row>
     <row r="21" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="n">
         <f aca="false">A20+TIME(0,30,0)</f>
         <v>1.10416666666667</v>
       </c>
-      <c r="B21" s="3" t="n">
+      <c r="B21" s="4" t="n">
         <f aca="false">A21+TIME(0,$Q$1,0)</f>
         <v>1.125</v>
       </c>
-      <c r="C21" s="4"/>
-      <c r="D21" s="4"/>
-      <c r="E21" s="4"/>
-      <c r="F21" s="4"/>
-      <c r="G21" s="4"/>
-      <c r="I21" s="4"/>
-      <c r="J21" s="4"/>
-      <c r="K21" s="4"/>
+      <c r="C21" s="5"/>
+      <c r="D21" s="5"/>
+      <c r="E21" s="5"/>
+      <c r="F21" s="5"/>
+      <c r="G21" s="5"/>
+      <c r="H21" s="7"/>
+      <c r="I21" s="5"/>
+      <c r="J21" s="5"/>
+      <c r="K21" s="5"/>
     </row>
     <row r="22" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="n">
         <f aca="false">A21+TIME(0,30,0)</f>
         <v>1.125</v>
       </c>
-      <c r="B22" s="3" t="n">
+      <c r="B22" s="4" t="n">
         <f aca="false">A22+TIME(0,$Q$1,0)</f>
         <v>1.14583333333333</v>
       </c>
-      <c r="C22" s="4"/>
-      <c r="D22" s="4"/>
-      <c r="E22" s="4"/>
-      <c r="F22" s="4"/>
-      <c r="G22" s="4"/>
-      <c r="I22" s="4"/>
-      <c r="J22" s="4"/>
-      <c r="K22" s="4"/>
+      <c r="C22" s="5"/>
+      <c r="D22" s="5"/>
+      <c r="E22" s="5"/>
+      <c r="F22" s="5"/>
+      <c r="G22" s="5"/>
+      <c r="H22" s="7"/>
+      <c r="I22" s="5"/>
+      <c r="J22" s="5"/>
+      <c r="K22" s="5"/>
     </row>
     <row r="23" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="n">
         <f aca="false">A22+TIME(0,30,0)</f>
         <v>1.14583333333333</v>
       </c>
-      <c r="B23" s="3" t="n">
+      <c r="B23" s="4" t="n">
         <f aca="false">A23+TIME(0,$Q$1,0)</f>
         <v>1.16666666666667</v>
       </c>
-      <c r="C23" s="4"/>
-      <c r="D23" s="4"/>
-      <c r="E23" s="4"/>
-      <c r="F23" s="4"/>
-      <c r="G23" s="4"/>
-      <c r="I23" s="4"/>
-      <c r="J23" s="4"/>
-      <c r="K23" s="4"/>
+      <c r="C23" s="5"/>
+      <c r="D23" s="5"/>
+      <c r="E23" s="5"/>
+      <c r="F23" s="5"/>
+      <c r="G23" s="5"/>
+      <c r="H23" s="7"/>
+      <c r="I23" s="5"/>
+      <c r="J23" s="5"/>
+      <c r="K23" s="5"/>
     </row>
     <row r="24" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="n">
         <f aca="false">A23+TIME(0,30,0)</f>
         <v>1.16666666666667</v>
       </c>
-      <c r="B24" s="3" t="n">
+      <c r="B24" s="4" t="n">
         <f aca="false">A24+TIME(0,$Q$1,0)</f>
         <v>1.1875</v>
       </c>
-      <c r="C24" s="4" t="s">
+      <c r="C24" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="D24" s="4"/>
-      <c r="E24" s="4"/>
-      <c r="F24" s="4" t="s">
+      <c r="D24" s="5"/>
+      <c r="E24" s="5"/>
+      <c r="F24" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="G24" s="4"/>
-      <c r="H24" s="4"/>
-      <c r="I24" s="4" t="s">
+      <c r="G24" s="5"/>
+      <c r="H24" s="5"/>
+      <c r="I24" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="J24" s="4"/>
-      <c r="K24" s="4"/>
+      <c r="J24" s="5"/>
+      <c r="K24" s="5"/>
     </row>
     <row r="25" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B25" s="3"/>
+      <c r="B25" s="4"/>
     </row>
     <row r="26" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="27" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -1022,50 +1044,50 @@
     <row r="33" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="34" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="35" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C35" s="6"/>
-      <c r="D35" s="6"/>
-      <c r="F35" s="2"/>
-      <c r="I35" s="2"/>
-      <c r="L35" s="2"/>
+      <c r="C35" s="8"/>
+      <c r="D35" s="8"/>
+      <c r="F35" s="3"/>
+      <c r="I35" s="3"/>
+      <c r="L35" s="3"/>
     </row>
     <row r="36" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C36" s="2"/>
-      <c r="F36" s="2"/>
-      <c r="L36" s="2"/>
+      <c r="C36" s="3"/>
+      <c r="F36" s="3"/>
+      <c r="L36" s="3"/>
     </row>
     <row r="37" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="38" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C38" s="2"/>
-      <c r="E38" s="7"/>
-      <c r="F38" s="2"/>
-      <c r="G38" s="2"/>
-      <c r="I38" s="2"/>
-      <c r="L38" s="2"/>
+      <c r="C38" s="3"/>
+      <c r="E38" s="9"/>
+      <c r="F38" s="3"/>
+      <c r="G38" s="3"/>
+      <c r="I38" s="3"/>
+      <c r="L38" s="3"/>
     </row>
     <row r="39" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C39" s="2"/>
-      <c r="D39" s="2"/>
+      <c r="C39" s="3"/>
+      <c r="D39" s="3"/>
     </row>
     <row r="40" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="F40" s="2"/>
-      <c r="I40" s="2"/>
+      <c r="F40" s="3"/>
+      <c r="I40" s="3"/>
     </row>
     <row r="41" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="I41" s="8"/>
-      <c r="K41" s="2"/>
+      <c r="I41" s="10"/>
+      <c r="K41" s="3"/>
     </row>
     <row r="42" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C42" s="2"/>
+      <c r="C42" s="3"/>
     </row>
     <row r="43" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="I43" s="2"/>
+      <c r="I43" s="3"/>
     </row>
     <row r="44" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="I44" s="2"/>
+      <c r="I44" s="3"/>
     </row>
     <row r="45" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="46" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C46" s="2"/>
+      <c r="C46" s="3"/>
     </row>
     <row r="47" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="48" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -2023,7 +2045,7 @@
     <row r="1000" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <mergeCells count="37">
+  <mergeCells count="38">
     <mergeCell ref="C1:E1"/>
     <mergeCell ref="F1:H1"/>
     <mergeCell ref="I1:K1"/>
@@ -2033,26 +2055,27 @@
     <mergeCell ref="E2:E3"/>
     <mergeCell ref="F2:G3"/>
     <mergeCell ref="H2:H3"/>
-    <mergeCell ref="I2:J7"/>
-    <mergeCell ref="K2:K7"/>
+    <mergeCell ref="I2:J4"/>
+    <mergeCell ref="K2:K4"/>
     <mergeCell ref="L2:M3"/>
     <mergeCell ref="N2:N3"/>
     <mergeCell ref="C4:E7"/>
-    <mergeCell ref="F4:G6"/>
+    <mergeCell ref="F4:H7"/>
     <mergeCell ref="L4:N7"/>
-    <mergeCell ref="F7:F8"/>
-    <mergeCell ref="G7:G8"/>
-    <mergeCell ref="H7:H11"/>
+    <mergeCell ref="I5:K8"/>
     <mergeCell ref="C8:C9"/>
     <mergeCell ref="D8:D9"/>
     <mergeCell ref="E8:E11"/>
-    <mergeCell ref="I8:J11"/>
+    <mergeCell ref="F8:F9"/>
+    <mergeCell ref="G8:G9"/>
+    <mergeCell ref="H8:H11"/>
     <mergeCell ref="L8:N15"/>
-    <mergeCell ref="F9:G23"/>
+    <mergeCell ref="I9:J13"/>
+    <mergeCell ref="K9:K13"/>
     <mergeCell ref="C10:C15"/>
     <mergeCell ref="D10:D15"/>
-    <mergeCell ref="K11:K13"/>
-    <mergeCell ref="I12:J13"/>
+    <mergeCell ref="F10:G23"/>
+    <mergeCell ref="H12:H23"/>
     <mergeCell ref="I14:J17"/>
     <mergeCell ref="K14:K17"/>
     <mergeCell ref="C16:E23"/>

</xml_diff>

<commit_message>
Updated programme and fixed some issues in the program.js
</commit_message>
<xml_diff>
--- a/programme-parser/programme.xlsx
+++ b/programme-parser/programme.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="35">
   <si>
     <t xml:space="preserve">Starttime</t>
   </si>
@@ -43,6 +43,12 @@
     <t xml:space="preserve">Resolution (min)</t>
   </si>
   <si>
+    <t xml:space="preserve">D&amp;D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chillûûûûh</t>
+  </si>
+  <si>
     <t xml:space="preserve">Megaspellen</t>
   </si>
   <si>
@@ -52,21 +58,15 @@
     <t xml:space="preserve">3D twister (VVT)</t>
   </si>
   <si>
-    <t xml:space="preserve">Arts and Crafts</t>
+    <t xml:space="preserve">BLÅHAKEN</t>
   </si>
   <si>
     <t xml:space="preserve">Escape Room (VVT)</t>
   </si>
   <si>
-    <t xml:space="preserve">D&amp;D</t>
-  </si>
-  <si>
     <t xml:space="preserve">Botter Rossen (VVT)</t>
   </si>
   <si>
-    <t xml:space="preserve">Chillûûûûh</t>
-  </si>
-  <si>
     <t xml:space="preserve">VVThee (VVT)</t>
   </si>
   <si>
@@ -85,25 +85,25 @@
     <t xml:space="preserve">Weerwolven</t>
   </si>
   <si>
+    <t xml:space="preserve">Sterrenkijken op de boot (VVT)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Band op de boot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kijken hoe het klinkt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deken is lava (VVT)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Retrogames</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spelletjesavond</t>
+  </si>
+  <si>
     <t xml:space="preserve">Preimeppen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sterrenkijken (VVT)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Band op de boot</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kijken hoe het klinkt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Deken is lava (VVT)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Retrogames</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Spelletjesavond</t>
   </si>
   <si>
     <t xml:space="preserve">Karaoke cocktailnight</t>
@@ -208,7 +208,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -231,10 +231,6 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -442,7 +438,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:Q1048576"/>
+  <dimension ref="A1:Q1002"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="1" width="11.5"/>
@@ -488,102 +484,96 @@
     </row>
     <row r="2" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="n">
-        <f aca="false">TIME(17,0,0)</f>
-        <v>0.708333333333333</v>
+        <f aca="false">TIME(16,0,0)</f>
+        <v>0.666666666666667</v>
       </c>
       <c r="B2" s="4" t="n">
         <f aca="false">A2+TIME(0,$Q$1,0)</f>
-        <v>0.729166666666667</v>
-      </c>
-      <c r="C2" s="5" t="s">
+        <v>0.6875</v>
+      </c>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="J2" s="3"/>
+      <c r="K2" s="3"/>
+      <c r="L2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="G2" s="5"/>
-      <c r="H2" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="I2" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="J2" s="5"/>
-      <c r="K2" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="L2" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="M2" s="5"/>
-      <c r="N2" s="5" t="s">
-        <v>15</v>
-      </c>
+      <c r="M2" s="3"/>
+      <c r="N2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="n">
         <f aca="false">A2+TIME(0,$Q$1,0)</f>
-        <v>0.729166666666667</v>
+        <v>0.6875</v>
       </c>
       <c r="B3" s="4" t="n">
         <f aca="false">A3+TIME(0,$Q$1,0)</f>
-        <v>0.75</v>
-      </c>
-      <c r="C3" s="5"/>
-      <c r="D3" s="5"/>
-      <c r="E3" s="5"/>
-      <c r="F3" s="5"/>
-      <c r="G3" s="5"/>
-      <c r="H3" s="5"/>
-      <c r="I3" s="5"/>
-      <c r="J3" s="5"/>
-      <c r="K3" s="5"/>
-      <c r="L3" s="5"/>
-      <c r="M3" s="5"/>
-      <c r="N3" s="5"/>
+        <v>0.708333333333333</v>
+      </c>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
+      <c r="J3" s="3"/>
+      <c r="K3" s="3"/>
+      <c r="L3" s="3"/>
+      <c r="M3" s="3"/>
+      <c r="N3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="n">
-        <f aca="false">A3+TIME(0,30,0)</f>
-        <v>0.75</v>
+        <f aca="false">A3+TIME(0,$Q$1,0)</f>
+        <v>0.708333333333333</v>
       </c>
       <c r="B4" s="4" t="n">
         <f aca="false">A4+TIME(0,$Q$1,0)</f>
-        <v>0.770833333333333</v>
+        <v>0.729166666666667</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
+        <v>9</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>11</v>
+      </c>
       <c r="F4" s="5" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="G4" s="5"/>
-      <c r="H4" s="5"/>
-      <c r="I4" s="5"/>
-      <c r="J4" s="5"/>
-      <c r="K4" s="5"/>
-      <c r="L4" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="M4" s="5"/>
-      <c r="N4" s="5"/>
+      <c r="H4" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="I4" s="3"/>
+      <c r="J4" s="3"/>
+      <c r="K4" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="L4" s="3"/>
+      <c r="M4" s="3"/>
+      <c r="N4" s="5" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="n">
-        <f aca="false">A4+TIME(0,30,0)</f>
-        <v>0.770833333333333</v>
+        <f aca="false">A4+TIME(0,$Q$1,0)</f>
+        <v>0.729166666666667</v>
       </c>
       <c r="B5" s="4" t="n">
         <f aca="false">A5+TIME(0,$Q$1,0)</f>
-        <v>0.791666666666667</v>
+        <v>0.75</v>
       </c>
       <c r="C5" s="5"/>
       <c r="D5" s="5"/>
@@ -591,45 +581,49 @@
       <c r="F5" s="5"/>
       <c r="G5" s="5"/>
       <c r="H5" s="5"/>
-      <c r="I5" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="J5" s="5"/>
+      <c r="I5" s="3"/>
+      <c r="J5" s="3"/>
       <c r="K5" s="5"/>
-      <c r="L5" s="5"/>
-      <c r="M5" s="5"/>
+      <c r="L5" s="3"/>
+      <c r="M5" s="3"/>
       <c r="N5" s="5"/>
     </row>
     <row r="6" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="n">
         <f aca="false">A5+TIME(0,30,0)</f>
-        <v>0.791666666666667</v>
+        <v>0.75</v>
       </c>
       <c r="B6" s="4" t="n">
         <f aca="false">A6+TIME(0,$Q$1,0)</f>
-        <v>0.8125</v>
-      </c>
-      <c r="C6" s="5"/>
+        <v>0.770833333333333</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>16</v>
+      </c>
       <c r="D6" s="5"/>
       <c r="E6" s="5"/>
-      <c r="F6" s="5"/>
+      <c r="F6" s="5" t="s">
+        <v>16</v>
+      </c>
       <c r="G6" s="5"/>
       <c r="H6" s="5"/>
-      <c r="I6" s="5"/>
-      <c r="J6" s="5"/>
+      <c r="I6" s="3"/>
+      <c r="J6" s="3"/>
       <c r="K6" s="5"/>
-      <c r="L6" s="5"/>
+      <c r="L6" s="5" t="s">
+        <v>16</v>
+      </c>
       <c r="M6" s="5"/>
       <c r="N6" s="5"/>
     </row>
     <row r="7" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="n">
         <f aca="false">A6+TIME(0,30,0)</f>
-        <v>0.8125</v>
+        <v>0.770833333333333</v>
       </c>
       <c r="B7" s="4" t="n">
         <f aca="false">A7+TIME(0,$Q$1,0)</f>
-        <v>0.833333333333333</v>
+        <v>0.791666666666667</v>
       </c>
       <c r="C7" s="5"/>
       <c r="D7" s="5"/>
@@ -637,7 +631,9 @@
       <c r="F7" s="5"/>
       <c r="G7" s="5"/>
       <c r="H7" s="5"/>
-      <c r="I7" s="5"/>
+      <c r="I7" s="5" t="s">
+        <v>16</v>
+      </c>
       <c r="J7" s="5"/>
       <c r="K7" s="5"/>
       <c r="L7" s="5"/>
@@ -647,47 +643,33 @@
     <row r="8" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="n">
         <f aca="false">A7+TIME(0,30,0)</f>
-        <v>0.833333333333333</v>
+        <v>0.791666666666667</v>
       </c>
       <c r="B8" s="4" t="n">
         <f aca="false">A8+TIME(0,$Q$1,0)</f>
-        <v>0.854166666666667</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="G8" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="H8" s="5" t="s">
-        <v>22</v>
-      </c>
+        <v>0.8125</v>
+      </c>
+      <c r="C8" s="5"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="5"/>
+      <c r="F8" s="5"/>
+      <c r="G8" s="5"/>
+      <c r="H8" s="5"/>
       <c r="I8" s="5"/>
       <c r="J8" s="5"/>
       <c r="K8" s="5"/>
-      <c r="L8" s="5" t="s">
-        <v>23</v>
-      </c>
+      <c r="L8" s="5"/>
       <c r="M8" s="5"/>
       <c r="N8" s="5"/>
     </row>
     <row r="9" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="n">
         <f aca="false">A8+TIME(0,30,0)</f>
-        <v>0.854166666666667</v>
+        <v>0.8125</v>
       </c>
       <c r="B9" s="4" t="n">
         <f aca="false">A9+TIME(0,$Q$1,0)</f>
-        <v>0.875</v>
+        <v>0.833333333333333</v>
       </c>
       <c r="C9" s="5"/>
       <c r="D9" s="5"/>
@@ -695,13 +677,9 @@
       <c r="F9" s="5"/>
       <c r="G9" s="5"/>
       <c r="H9" s="5"/>
-      <c r="I9" s="5" t="s">
-        <v>24</v>
-      </c>
+      <c r="I9" s="5"/>
       <c r="J9" s="5"/>
-      <c r="K9" s="6" t="s">
-        <v>25</v>
-      </c>
+      <c r="K9" s="5"/>
       <c r="L9" s="5"/>
       <c r="M9" s="5"/>
       <c r="N9" s="5"/>
@@ -709,39 +687,45 @@
     <row r="10" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="n">
         <f aca="false">A9+TIME(0,30,0)</f>
-        <v>0.875</v>
+        <v>0.833333333333333</v>
       </c>
       <c r="B10" s="4" t="n">
         <f aca="false">A10+TIME(0,$Q$1,0)</f>
-        <v>0.895833333333333</v>
+        <v>0.854166666666667</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="E10" s="5"/>
+        <v>18</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="F10" s="5" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="G10" s="5"/>
-      <c r="H10" s="5"/>
+      <c r="H10" s="5" t="s">
+        <v>21</v>
+      </c>
       <c r="I10" s="5"/>
       <c r="J10" s="5"/>
-      <c r="K10" s="6"/>
-      <c r="L10" s="5"/>
+      <c r="K10" s="5"/>
+      <c r="L10" s="5" t="s">
+        <v>22</v>
+      </c>
       <c r="M10" s="5"/>
       <c r="N10" s="5"/>
     </row>
     <row r="11" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="n">
         <f aca="false">A10+TIME(0,30,0)</f>
-        <v>0.895833333333333</v>
+        <v>0.854166666666667</v>
       </c>
       <c r="B11" s="4" t="n">
         <f aca="false">A11+TIME(0,$Q$1,0)</f>
-        <v>0.916666666666667</v>
+        <v>0.875</v>
       </c>
       <c r="C11" s="5"/>
       <c r="D11" s="5"/>
@@ -749,9 +733,13 @@
       <c r="F11" s="5"/>
       <c r="G11" s="5"/>
       <c r="H11" s="5"/>
-      <c r="I11" s="5"/>
+      <c r="I11" s="5" t="s">
+        <v>23</v>
+      </c>
       <c r="J11" s="5"/>
-      <c r="K11" s="6"/>
+      <c r="K11" s="6" t="s">
+        <v>24</v>
+      </c>
       <c r="L11" s="5"/>
       <c r="M11" s="5"/>
       <c r="N11" s="5"/>
@@ -759,19 +747,24 @@
     <row r="12" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="n">
         <f aca="false">A11+TIME(0,30,0)</f>
-        <v>0.916666666666667</v>
+        <v>0.875</v>
       </c>
       <c r="B12" s="4" t="n">
         <f aca="false">A12+TIME(0,$Q$1,0)</f>
-        <v>0.9375</v>
-      </c>
-      <c r="C12" s="5"/>
-      <c r="D12" s="5"/>
-      <c r="F12" s="5"/>
+        <v>0.895833333333333</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="E12" s="5"/>
+      <c r="F12" s="5" t="s">
+        <v>27</v>
+      </c>
       <c r="G12" s="5"/>
-      <c r="H12" s="7" t="s">
-        <v>28</v>
-      </c>
+      <c r="H12" s="5"/>
       <c r="I12" s="5"/>
       <c r="J12" s="5"/>
       <c r="K12" s="6"/>
@@ -782,17 +775,18 @@
     <row r="13" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="n">
         <f aca="false">A12+TIME(0,30,0)</f>
-        <v>0.9375</v>
+        <v>0.895833333333333</v>
       </c>
       <c r="B13" s="4" t="n">
         <f aca="false">A13+TIME(0,$Q$1,0)</f>
-        <v>0.958333333333333</v>
+        <v>0.916666666666667</v>
       </c>
       <c r="C13" s="5"/>
       <c r="D13" s="5"/>
+      <c r="E13" s="5"/>
       <c r="F13" s="5"/>
       <c r="G13" s="5"/>
-      <c r="H13" s="7"/>
+      <c r="H13" s="5"/>
       <c r="I13" s="5"/>
       <c r="J13" s="5"/>
       <c r="K13" s="6"/>
@@ -803,24 +797,24 @@
     <row r="14" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="n">
         <f aca="false">A13+TIME(0,30,0)</f>
-        <v>0.958333333333333</v>
+        <v>0.916666666666667</v>
       </c>
       <c r="B14" s="4" t="n">
         <f aca="false">A14+TIME(0,$Q$1,0)</f>
-        <v>0.979166666666667</v>
+        <v>0.9375</v>
       </c>
       <c r="C14" s="5"/>
       <c r="D14" s="5"/>
-      <c r="F14" s="5"/>
+      <c r="F14" s="5" t="s">
+        <v>28</v>
+      </c>
       <c r="G14" s="5"/>
-      <c r="H14" s="7"/>
+      <c r="H14" s="5"/>
       <c r="I14" s="5" t="s">
         <v>29</v>
       </c>
       <c r="J14" s="5"/>
-      <c r="K14" s="5" t="s">
-        <v>30</v>
-      </c>
+      <c r="K14" s="6"/>
       <c r="L14" s="5"/>
       <c r="M14" s="5"/>
       <c r="N14" s="5"/>
@@ -828,20 +822,20 @@
     <row r="15" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="n">
         <f aca="false">A14+TIME(0,30,0)</f>
-        <v>0.979166666666667</v>
+        <v>0.9375</v>
       </c>
       <c r="B15" s="4" t="n">
         <f aca="false">A15+TIME(0,$Q$1,0)</f>
-        <v>1</v>
+        <v>0.958333333333333</v>
       </c>
       <c r="C15" s="5"/>
       <c r="D15" s="5"/>
       <c r="F15" s="5"/>
       <c r="G15" s="5"/>
-      <c r="H15" s="7"/>
+      <c r="H15" s="5"/>
       <c r="I15" s="5"/>
       <c r="J15" s="5"/>
-      <c r="K15" s="5"/>
+      <c r="K15" s="6"/>
       <c r="L15" s="5"/>
       <c r="M15" s="5"/>
       <c r="N15" s="5"/>
@@ -849,138 +843,144 @@
     <row r="16" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="n">
         <f aca="false">A15+TIME(0,30,0)</f>
-        <v>1</v>
+        <v>0.958333333333333</v>
       </c>
       <c r="B16" s="4" t="n">
         <f aca="false">A16+TIME(0,$Q$1,0)</f>
-        <v>1.02083333333333</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>31</v>
-      </c>
+        <v>0.979166666666667</v>
+      </c>
+      <c r="C16" s="5"/>
       <c r="D16" s="5"/>
-      <c r="E16" s="5"/>
       <c r="F16" s="5"/>
       <c r="G16" s="5"/>
-      <c r="H16" s="7"/>
+      <c r="H16" s="5"/>
       <c r="I16" s="5"/>
       <c r="J16" s="5"/>
-      <c r="K16" s="5"/>
+      <c r="K16" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="L16" s="5"/>
+      <c r="M16" s="5"/>
+      <c r="N16" s="5"/>
     </row>
     <row r="17" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="n">
         <f aca="false">A16+TIME(0,30,0)</f>
-        <v>1.02083333333333</v>
+        <v>0.979166666666667</v>
       </c>
       <c r="B17" s="4" t="n">
         <f aca="false">A17+TIME(0,$Q$1,0)</f>
-        <v>1.04166666666667</v>
+        <v>1</v>
       </c>
       <c r="C17" s="5"/>
       <c r="D17" s="5"/>
-      <c r="E17" s="5"/>
       <c r="F17" s="5"/>
       <c r="G17" s="5"/>
-      <c r="H17" s="7"/>
+      <c r="H17" s="5"/>
       <c r="I17" s="5"/>
       <c r="J17" s="5"/>
       <c r="K17" s="5"/>
+      <c r="L17" s="5"/>
+      <c r="M17" s="5"/>
+      <c r="N17" s="5"/>
     </row>
     <row r="18" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="n">
         <f aca="false">A17+TIME(0,30,0)</f>
-        <v>1.04166666666667</v>
+        <v>1</v>
       </c>
       <c r="B18" s="4" t="n">
         <f aca="false">A18+TIME(0,$Q$1,0)</f>
-        <v>1.0625</v>
-      </c>
-      <c r="C18" s="5"/>
+        <v>1.02083333333333</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>31</v>
+      </c>
       <c r="D18" s="5"/>
       <c r="E18" s="5"/>
       <c r="F18" s="5"/>
       <c r="G18" s="5"/>
-      <c r="H18" s="7"/>
-      <c r="I18" s="5" t="s">
-        <v>32</v>
-      </c>
+      <c r="H18" s="5"/>
+      <c r="I18" s="5"/>
       <c r="J18" s="5"/>
       <c r="K18" s="5"/>
     </row>
     <row r="19" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="n">
         <f aca="false">A18+TIME(0,30,0)</f>
-        <v>1.0625</v>
+        <v>1.02083333333333</v>
       </c>
       <c r="B19" s="4" t="n">
         <f aca="false">A19+TIME(0,$Q$1,0)</f>
-        <v>1.08333333333333</v>
+        <v>1.04166666666667</v>
       </c>
       <c r="C19" s="5"/>
       <c r="D19" s="5"/>
       <c r="E19" s="5"/>
       <c r="F19" s="5"/>
       <c r="G19" s="5"/>
-      <c r="H19" s="7"/>
-      <c r="I19" s="5" t="s">
-        <v>33</v>
-      </c>
+      <c r="H19" s="5"/>
+      <c r="I19" s="5"/>
       <c r="J19" s="5"/>
       <c r="K19" s="5"/>
     </row>
     <row r="20" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="n">
         <f aca="false">A19+TIME(0,30,0)</f>
-        <v>1.08333333333333</v>
+        <v>1.04166666666667</v>
       </c>
       <c r="B20" s="4" t="n">
         <f aca="false">A20+TIME(0,$Q$1,0)</f>
-        <v>1.10416666666667</v>
+        <v>1.0625</v>
       </c>
       <c r="C20" s="5"/>
       <c r="D20" s="5"/>
       <c r="E20" s="5"/>
       <c r="F20" s="5"/>
       <c r="G20" s="5"/>
-      <c r="H20" s="7"/>
-      <c r="I20" s="5"/>
+      <c r="H20" s="5"/>
+      <c r="I20" s="5" t="s">
+        <v>32</v>
+      </c>
       <c r="J20" s="5"/>
       <c r="K20" s="5"/>
     </row>
     <row r="21" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="n">
         <f aca="false">A20+TIME(0,30,0)</f>
-        <v>1.10416666666667</v>
+        <v>1.0625</v>
       </c>
       <c r="B21" s="4" t="n">
         <f aca="false">A21+TIME(0,$Q$1,0)</f>
-        <v>1.125</v>
+        <v>1.08333333333333</v>
       </c>
       <c r="C21" s="5"/>
       <c r="D21" s="5"/>
       <c r="E21" s="5"/>
       <c r="F21" s="5"/>
       <c r="G21" s="5"/>
-      <c r="H21" s="7"/>
-      <c r="I21" s="5"/>
+      <c r="H21" s="5"/>
+      <c r="I21" s="5" t="s">
+        <v>33</v>
+      </c>
       <c r="J21" s="5"/>
       <c r="K21" s="5"/>
     </row>
     <row r="22" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="n">
         <f aca="false">A21+TIME(0,30,0)</f>
-        <v>1.125</v>
+        <v>1.08333333333333</v>
       </c>
       <c r="B22" s="4" t="n">
         <f aca="false">A22+TIME(0,$Q$1,0)</f>
-        <v>1.14583333333333</v>
+        <v>1.10416666666667</v>
       </c>
       <c r="C22" s="5"/>
       <c r="D22" s="5"/>
       <c r="E22" s="5"/>
       <c r="F22" s="5"/>
       <c r="G22" s="5"/>
-      <c r="H22" s="7"/>
+      <c r="H22" s="5"/>
       <c r="I22" s="5"/>
       <c r="J22" s="5"/>
       <c r="K22" s="5"/>
@@ -988,18 +988,18 @@
     <row r="23" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="n">
         <f aca="false">A22+TIME(0,30,0)</f>
-        <v>1.14583333333333</v>
+        <v>1.10416666666667</v>
       </c>
       <c r="B23" s="4" t="n">
         <f aca="false">A23+TIME(0,$Q$1,0)</f>
-        <v>1.16666666666667</v>
+        <v>1.125</v>
       </c>
       <c r="C23" s="5"/>
       <c r="D23" s="5"/>
       <c r="E23" s="5"/>
       <c r="F23" s="5"/>
       <c r="G23" s="5"/>
-      <c r="H23" s="7"/>
+      <c r="H23" s="5"/>
       <c r="I23" s="5"/>
       <c r="J23" s="5"/>
       <c r="K23" s="5"/>
@@ -1007,90 +1007,126 @@
     <row r="24" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="n">
         <f aca="false">A23+TIME(0,30,0)</f>
-        <v>1.16666666666667</v>
+        <v>1.125</v>
       </c>
       <c r="B24" s="4" t="n">
         <f aca="false">A24+TIME(0,$Q$1,0)</f>
-        <v>1.1875</v>
-      </c>
-      <c r="C24" s="5" t="s">
-        <v>34</v>
-      </c>
+        <v>1.14583333333333</v>
+      </c>
+      <c r="C24" s="5"/>
       <c r="D24" s="5"/>
       <c r="E24" s="5"/>
-      <c r="F24" s="5" t="s">
-        <v>34</v>
-      </c>
+      <c r="F24" s="5"/>
       <c r="G24" s="5"/>
       <c r="H24" s="5"/>
-      <c r="I24" s="5" t="s">
-        <v>34</v>
-      </c>
+      <c r="I24" s="5"/>
       <c r="J24" s="5"/>
       <c r="K24" s="5"/>
     </row>
     <row r="25" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B25" s="4"/>
-    </row>
-    <row r="26" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="27" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+      <c r="A25" s="1" t="n">
+        <f aca="false">A24+TIME(0,30,0)</f>
+        <v>1.14583333333333</v>
+      </c>
+      <c r="B25" s="4" t="n">
+        <f aca="false">A25+TIME(0,$Q$1,0)</f>
+        <v>1.16666666666667</v>
+      </c>
+      <c r="C25" s="5"/>
+      <c r="D25" s="5"/>
+      <c r="E25" s="5"/>
+      <c r="F25" s="5"/>
+      <c r="G25" s="5"/>
+      <c r="H25" s="5"/>
+      <c r="I25" s="5"/>
+      <c r="J25" s="5"/>
+      <c r="K25" s="5"/>
+    </row>
+    <row r="26" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="1" t="n">
+        <f aca="false">A25+TIME(0,30,0)</f>
+        <v>1.16666666666667</v>
+      </c>
+      <c r="B26" s="4" t="n">
+        <f aca="false">A26+TIME(0,$Q$1,0)</f>
+        <v>1.1875</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="D26" s="5"/>
+      <c r="E26" s="5"/>
+      <c r="F26" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="G26" s="5"/>
+      <c r="H26" s="5"/>
+      <c r="I26" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="J26" s="5"/>
+      <c r="K26" s="5"/>
+    </row>
+    <row r="27" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B27" s="4"/>
+    </row>
     <row r="28" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="29" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="30" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="31" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="O31" s="1"/>
-    </row>
+    <row r="31" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="32" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="33" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="33" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="O33" s="1"/>
+    </row>
     <row r="34" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="35" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C35" s="8"/>
-      <c r="D35" s="8"/>
-      <c r="F35" s="3"/>
-      <c r="I35" s="3"/>
-      <c r="L35" s="3"/>
-    </row>
-    <row r="36" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C36" s="3"/>
-      <c r="F36" s="3"/>
-      <c r="L36" s="3"/>
-    </row>
-    <row r="37" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="35" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="36" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="37" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C37" s="7"/>
+      <c r="D37" s="7"/>
+      <c r="F37" s="3"/>
+      <c r="I37" s="3"/>
+      <c r="L37" s="3"/>
+    </row>
     <row r="38" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C38" s="3"/>
-      <c r="E38" s="9"/>
       <c r="F38" s="3"/>
-      <c r="G38" s="3"/>
-      <c r="I38" s="3"/>
       <c r="L38" s="3"/>
     </row>
-    <row r="39" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C39" s="3"/>
-      <c r="D39" s="3"/>
-    </row>
+    <row r="39" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="40" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C40" s="3"/>
+      <c r="E40" s="8"/>
       <c r="F40" s="3"/>
+      <c r="G40" s="3"/>
       <c r="I40" s="3"/>
+      <c r="L40" s="3"/>
     </row>
     <row r="41" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="I41" s="10"/>
-      <c r="K41" s="3"/>
+      <c r="C41" s="3"/>
+      <c r="D41" s="3"/>
     </row>
     <row r="42" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C42" s="3"/>
+      <c r="F42" s="3"/>
+      <c r="I42" s="3"/>
     </row>
     <row r="43" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="I43" s="3"/>
+      <c r="I43" s="9"/>
+      <c r="K43" s="3"/>
     </row>
     <row r="44" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="I44" s="3"/>
-    </row>
-    <row r="45" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+      <c r="C44" s="3"/>
+    </row>
+    <row r="45" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="I45" s="3"/>
+    </row>
     <row r="46" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C46" s="3"/>
+      <c r="I46" s="3"/>
     </row>
     <row r="47" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="48" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="48" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C48" s="3"/>
+    </row>
     <row r="49" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="50" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="51" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -2043,47 +2079,47 @@
     <row r="998" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="999" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="1000" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1001" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1002" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <mergeCells count="38">
+  <mergeCells count="37">
     <mergeCell ref="C1:E1"/>
     <mergeCell ref="F1:H1"/>
     <mergeCell ref="I1:K1"/>
     <mergeCell ref="L1:N1"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="D2:D3"/>
-    <mergeCell ref="E2:E3"/>
-    <mergeCell ref="F2:G3"/>
-    <mergeCell ref="H2:H3"/>
-    <mergeCell ref="I2:J4"/>
-    <mergeCell ref="K2:K4"/>
-    <mergeCell ref="L2:M3"/>
-    <mergeCell ref="N2:N3"/>
-    <mergeCell ref="C4:E7"/>
-    <mergeCell ref="F4:H7"/>
-    <mergeCell ref="L4:N7"/>
-    <mergeCell ref="I5:K8"/>
-    <mergeCell ref="C8:C9"/>
-    <mergeCell ref="D8:D9"/>
-    <mergeCell ref="E8:E11"/>
-    <mergeCell ref="F8:F9"/>
-    <mergeCell ref="G8:G9"/>
-    <mergeCell ref="H8:H11"/>
-    <mergeCell ref="L8:N15"/>
-    <mergeCell ref="I9:J13"/>
-    <mergeCell ref="K9:K13"/>
-    <mergeCell ref="C10:C15"/>
-    <mergeCell ref="D10:D15"/>
-    <mergeCell ref="F10:G23"/>
-    <mergeCell ref="H12:H23"/>
+    <mergeCell ref="I2:J6"/>
+    <mergeCell ref="L2:M5"/>
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="D4:D5"/>
+    <mergeCell ref="E4:E5"/>
+    <mergeCell ref="F4:G5"/>
+    <mergeCell ref="H4:H5"/>
+    <mergeCell ref="K4:K6"/>
+    <mergeCell ref="N4:N5"/>
+    <mergeCell ref="C6:E9"/>
+    <mergeCell ref="F6:H9"/>
+    <mergeCell ref="L6:N9"/>
+    <mergeCell ref="I7:K10"/>
+    <mergeCell ref="C10:C11"/>
+    <mergeCell ref="D10:D11"/>
+    <mergeCell ref="E10:E13"/>
+    <mergeCell ref="F10:G11"/>
+    <mergeCell ref="H10:H13"/>
+    <mergeCell ref="L10:N17"/>
+    <mergeCell ref="I11:J13"/>
+    <mergeCell ref="K11:K15"/>
+    <mergeCell ref="C12:C17"/>
+    <mergeCell ref="D12:D17"/>
+    <mergeCell ref="F12:G13"/>
+    <mergeCell ref="F14:H25"/>
     <mergeCell ref="I14:J17"/>
-    <mergeCell ref="K14:K17"/>
-    <mergeCell ref="C16:E23"/>
-    <mergeCell ref="I18:K18"/>
-    <mergeCell ref="I19:K23"/>
-    <mergeCell ref="C24:E24"/>
-    <mergeCell ref="F24:H24"/>
-    <mergeCell ref="I24:K24"/>
+    <mergeCell ref="K16:K19"/>
+    <mergeCell ref="C18:E25"/>
+    <mergeCell ref="I20:K20"/>
+    <mergeCell ref="I21:K25"/>
+    <mergeCell ref="C26:E26"/>
+    <mergeCell ref="F26:H26"/>
+    <mergeCell ref="I26:K26"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="0.7875" bottom="0.7875" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>